<commit_message>
Update documentation for Sprint 05 and Sprint 06, including adjustments to planned vs. actual metrics, retrospective details, and test execution reports. Corrected dates and improved formatting for clarity. Added summaries of completed tasks and commitments for better tracking of progress.
</commit_message>
<xml_diff>
--- a/Documentos Base/Sprint 4 documentacion/Sprint_04_Backlog_ICARO.xlsx
+++ b/Documentos Base/Sprint 4 documentacion/Sprint_04_Backlog_ICARO.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3043EBB9-4AC4-4DEF-83F9-D326ACE05761}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog Sprint 04" sheetId="4" r:id="rId1"/>
@@ -667,36 +667,9 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -714,20 +687,47 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1042,424 +1042,424 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="26" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="12" t="s">
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="H3" s="29">
+      <c r="H3" s="19">
         <v>4</v>
       </c>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
-      <c r="L3" s="31"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="21"/>
     </row>
     <row r="4" spans="1:12" ht="24" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="16">
+      <c r="B4" s="27">
         <v>46116</v>
       </c>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="12" t="s">
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="H4" s="16">
+      <c r="H4" s="27">
         <v>46150</v>
       </c>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="18"/>
+      <c r="I4" s="28"/>
+      <c r="J4" s="28"/>
+      <c r="K4" s="28"/>
+      <c r="L4" s="29"/>
     </row>
     <row r="5" spans="1:12" ht="95.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="12" t="s">
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="H5" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="15"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+      <c r="K5" s="17"/>
+      <c r="L5" s="18"/>
     </row>
     <row r="6" spans="1:12" ht="24" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="29">
+      <c r="B6" s="19">
         <v>22</v>
       </c>
-      <c r="C6" s="30"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="12" t="s">
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="14"/>
-      <c r="L6" s="15"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="18"/>
     </row>
     <row r="7" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="H7" s="19" t="s">
+      <c r="H7" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="I7" s="19" t="s">
+      <c r="I7" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="J7" s="19" t="s">
+      <c r="J7" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="K7" s="19" t="s">
+      <c r="K7" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="L7" s="19" t="s">
+      <c r="L7" s="8" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="126.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F8" s="20">
+      <c r="F8" s="9">
         <v>5</v>
       </c>
-      <c r="G8" s="20">
+      <c r="G8" s="9">
         <v>5</v>
       </c>
-      <c r="H8" s="21" t="s">
+      <c r="H8" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="I8" s="22" t="s">
+      <c r="I8" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="J8" s="21" t="s">
+      <c r="J8" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="K8" s="21" t="s">
+      <c r="K8" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="L8" s="21" t="s">
+      <c r="L8" s="10" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="96.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="23" t="s">
+      <c r="A9" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="23">
+      <c r="F9" s="12">
         <v>3</v>
       </c>
-      <c r="G9" s="23">
+      <c r="G9" s="12">
         <v>3</v>
       </c>
-      <c r="H9" s="21" t="s">
+      <c r="H9" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="I9" s="22" t="s">
+      <c r="I9" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="J9" s="24" t="s">
+      <c r="J9" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="K9" s="24" t="s">
+      <c r="K9" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="L9" s="24" t="s">
+      <c r="L9" s="13" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="120.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="D10" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="20" t="s">
+      <c r="E10" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="20">
+      <c r="F10" s="9">
         <v>2</v>
       </c>
-      <c r="G10" s="20">
+      <c r="G10" s="9">
         <v>2</v>
       </c>
-      <c r="H10" s="21" t="s">
+      <c r="H10" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="I10" s="22" t="s">
+      <c r="I10" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="J10" s="21" t="s">
+      <c r="J10" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="K10" s="21" t="s">
+      <c r="K10" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="L10" s="21" t="s">
+      <c r="L10" s="10" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="23" t="s">
+      <c r="A11" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="24" t="s">
+      <c r="D11" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="23" t="s">
+      <c r="E11" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="F11" s="23">
+      <c r="F11" s="12">
         <v>5</v>
       </c>
-      <c r="G11" s="23">
+      <c r="G11" s="12">
         <v>5</v>
       </c>
-      <c r="H11" s="21" t="s">
+      <c r="H11" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="I11" s="22" t="s">
+      <c r="I11" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="J11" s="24" t="s">
+      <c r="J11" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="K11" s="24" t="s">
+      <c r="K11" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="L11" s="24" t="s">
+      <c r="L11" s="13" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="119.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="20" t="s">
+      <c r="A12" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="21" t="s">
+      <c r="D12" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="20" t="s">
+      <c r="E12" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F12" s="20">
+      <c r="F12" s="9">
         <v>2</v>
       </c>
-      <c r="G12" s="20">
+      <c r="G12" s="9">
         <v>2</v>
       </c>
-      <c r="H12" s="21" t="s">
+      <c r="H12" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="I12" s="22" t="s">
+      <c r="I12" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="J12" s="21" t="s">
+      <c r="J12" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="K12" s="21" t="s">
+      <c r="K12" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="L12" s="21" t="s">
+      <c r="L12" s="10" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="117" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="23" t="s">
+      <c r="A13" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="D13" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="23" t="s">
+      <c r="E13" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="F13" s="23">
+      <c r="F13" s="12">
         <v>5</v>
       </c>
-      <c r="G13" s="23">
+      <c r="G13" s="12">
         <v>5</v>
       </c>
-      <c r="H13" s="21" t="s">
+      <c r="H13" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="I13" s="22" t="s">
+      <c r="I13" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="J13" s="24" t="s">
+      <c r="J13" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="K13" s="24" t="s">
+      <c r="K13" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="L13" s="24" t="s">
+      <c r="L13" s="13" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="25" t="s">
+      <c r="A14" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="26"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="27">
+      <c r="B14" s="23"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="15">
         <v>22</v>
       </c>
-      <c r="G14" s="27">
+      <c r="G14" s="15">
         <v>22</v>
       </c>
-      <c r="H14" s="28"/>
-      <c r="I14" s="28"/>
-      <c r="J14" s="28"/>
-      <c r="K14" s="28"/>
-      <c r="L14" s="28"/>
+      <c r="H14" s="14"/>
+      <c r="I14" s="14"/>
+      <c r="J14" s="14"/>
+      <c r="K14" s="14"/>
+      <c r="L14" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="H5:L5"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="H6:L6"/>
-    <mergeCell ref="A14:E14"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="H4:L4"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="H5:L5"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="H6:L6"/>
+    <mergeCell ref="A14:E14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1476,12 +1476,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1684,11 +1684,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">

</xml_diff>

<commit_message>
Cambios de sprint 4, 5,6,7
</commit_message>
<xml_diff>
--- a/Documentos Base/Sprint 4 documentacion/Sprint_04_Backlog_ICARO.xlsx
+++ b/Documentos Base/Sprint 4 documentacion/Sprint_04_Backlog_ICARO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hp\Desktop\Sistema_Gestion_Integral_Constructora\Documentos Base\Sprint 4 documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3043EBB9-4AC4-4DEF-83F9-D326ACE05761}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F988439-E337-4CEA-BE67-59FBA71F500F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog Sprint 04" sheetId="4" r:id="rId1"/>
@@ -363,9 +363,6 @@
     <t>Compromisos Sprint 03 8.3 cum.</t>
   </si>
   <si>
-    <t>SPRINT BACKLOG — Sprint 03: Catalogo de Materiales, Gestion de Bodega e Inventario</t>
-  </si>
-  <si>
     <t>ICARO CONSTRUCTORES BMGM S.A.S.  |  Sistema de Gestion Integral de Obra</t>
   </si>
   <si>
@@ -472,6 +469,9 @@
   </si>
   <si>
     <t>Implementar el módulo de Requerimientos de Compra con CRUD completo, registro de líneas de detalle, consulta por proyecto, filtros operativos, flujo de aprobación y rechazo con control RBAC, validación de justificación obligatoria para rechazos y formalización del endpoint de reactivación de materiales dados de baja. Adicionalmente, ampliar la cobertura de pruebas automatizadas sobre requerimientos de compra, aprobación/rechazo y reactivación de materiales</t>
+  </si>
+  <si>
+    <t>SPRINT BACKLOG — Sprint 04</t>
   </si>
 </sst>
 </file>
@@ -1043,7 +1043,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A1" s="24" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -1059,7 +1059,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
@@ -1085,7 +1085,7 @@
       <c r="E3" s="17"/>
       <c r="F3" s="18"/>
       <c r="G3" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H3" s="19">
         <v>4</v>
@@ -1107,7 +1107,7 @@
       <c r="E4" s="28"/>
       <c r="F4" s="29"/>
       <c r="G4" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H4" s="27">
         <v>46150</v>
@@ -1122,17 +1122,17 @@
         <v>3</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="17"/>
       <c r="E5" s="17"/>
       <c r="F5" s="18"/>
       <c r="G5" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="H5" s="16" t="s">
         <v>117</v>
-      </c>
-      <c r="H5" s="16" t="s">
-        <v>118</v>
       </c>
       <c r="I5" s="17"/>
       <c r="J5" s="17"/>
@@ -1151,10 +1151,10 @@
       <c r="E6" s="20"/>
       <c r="F6" s="21"/>
       <c r="G6" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="H6" s="16" t="s">
         <v>119</v>
-      </c>
-      <c r="H6" s="16" t="s">
-        <v>120</v>
       </c>
       <c r="I6" s="17"/>
       <c r="J6" s="17"/>
@@ -1181,22 +1181,22 @@
         <v>11</v>
       </c>
       <c r="G7" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="H7" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="I7" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="J7" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K7" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="J7" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="K7" s="8" t="s">
+      <c r="L7" s="8" t="s">
         <v>124</v>
-      </c>
-      <c r="L7" s="8" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="126.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1222,19 +1222,19 @@
         <v>5</v>
       </c>
       <c r="H8" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="I8" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="I8" s="11" t="s">
-        <v>127</v>
-      </c>
       <c r="J8" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="K8" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="K8" s="10" t="s">
+      <c r="L8" s="10" t="s">
         <v>130</v>
-      </c>
-      <c r="L8" s="10" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="96.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1242,7 +1242,7 @@
         <v>17</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>14</v>
@@ -1260,19 +1260,19 @@
         <v>3</v>
       </c>
       <c r="H9" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="I9" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="I9" s="11" t="s">
-        <v>127</v>
-      </c>
       <c r="J9" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="K9" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="K9" s="13" t="s">
+      <c r="L9" s="13" t="s">
         <v>134</v>
-      </c>
-      <c r="L9" s="13" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="120.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1298,19 +1298,19 @@
         <v>2</v>
       </c>
       <c r="H10" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="I10" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="I10" s="11" t="s">
-        <v>127</v>
-      </c>
       <c r="J10" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="K10" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="K10" s="10" t="s">
+      <c r="L10" s="10" t="s">
         <v>137</v>
-      </c>
-      <c r="L10" s="10" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1336,19 +1336,19 @@
         <v>5</v>
       </c>
       <c r="H11" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="I11" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="I11" s="11" t="s">
-        <v>127</v>
-      </c>
       <c r="J11" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="K11" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="K11" s="13" t="s">
+      <c r="L11" s="13" t="s">
         <v>140</v>
-      </c>
-      <c r="L11" s="13" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="119.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1356,7 +1356,7 @@
         <v>24</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>25</v>
@@ -1374,19 +1374,19 @@
         <v>2</v>
       </c>
       <c r="H12" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="I12" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="I12" s="11" t="s">
-        <v>127</v>
-      </c>
       <c r="J12" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="K12" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="K12" s="10" t="s">
+      <c r="L12" s="10" t="s">
         <v>144</v>
-      </c>
-      <c r="L12" s="10" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="117" customHeight="1" x14ac:dyDescent="0.25">
@@ -1412,19 +1412,19 @@
         <v>5</v>
       </c>
       <c r="H13" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="I13" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="I13" s="11" t="s">
-        <v>127</v>
-      </c>
       <c r="J13" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="K13" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="K13" s="13" t="s">
+      <c r="L13" s="13" t="s">
         <v>147</v>
-      </c>
-      <c r="L13" s="13" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>